<commit_message>
docs: ajouter les ID des 8 images générées au dossier de novembre
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FMRjbXSp29HtAam2YYiN3d
</commit_message>
<xml_diff>
--- a/docs/dossier-production-novembre-2026.xlsx
+++ b/docs/dossier-production-novembre-2026.xlsx
@@ -7732,7 +7732,7 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>À générer</t>
+          <t>Généré le 28/09 (Soul V2)</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -7740,7 +7740,11 @@
           <t>Devanture de commerce le soir, décorée pour Noël, sticker vierge sur la vitre</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr"/>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>bc0a40ea</t>
+        </is>
+      </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
           <t>généré</t>
@@ -7840,7 +7844,7 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>À générer</t>
+          <t>Généré le 28/09 (Soul V2)</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -7848,7 +7852,11 @@
           <t>Bûche de Noël dans sa boîte pâtissière ouverte, étiquette vierge</t>
         </is>
       </c>
-      <c r="E51" s="2" t="inlineStr"/>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>f8b0e3e7</t>
+        </is>
+      </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
           <t>généré</t>
@@ -8128,7 +8136,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>À générer</t>
+          <t>Généré le 28/09 (Soul V2)</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -8136,7 +8144,11 @@
           <t>Plateau de fruits de mer de fête sur glace, papier</t>
         </is>
       </c>
-      <c r="E59" s="2" t="inlineStr"/>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>c0a50f0f</t>
+        </is>
+      </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
           <t>généré</t>
@@ -8164,7 +8176,7 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>À générer</t>
+          <t>Généré le 28/09 (Soul V2)</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
@@ -8172,7 +8184,11 @@
           <t>Volaille de fête ficelée sur papier boucher</t>
         </is>
       </c>
-      <c r="E60" s="2" t="inlineStr"/>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>aa97dfff</t>
+        </is>
+      </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
           <t>généré</t>
@@ -8200,7 +8216,7 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>À générer</t>
+          <t>Généré le 28/09 (Soul V2)</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
@@ -8208,7 +8224,11 @@
           <t>Couronne de l'Avent sur l'établi du fleuriste</t>
         </is>
       </c>
-      <c r="E61" s="2" t="inlineStr"/>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>57b69978</t>
+        </is>
+      </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
           <t>généré</t>
@@ -8236,7 +8256,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>À générer</t>
+          <t>Généré le 28/09 (Soul V2)</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -8244,7 +8264,11 @@
           <t>Salle de restaurant le soir, table de 6 dressée et vide</t>
         </is>
       </c>
-      <c r="E62" s="2" t="inlineStr"/>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>dab06dad</t>
+        </is>
+      </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
           <t>généré</t>
@@ -8272,7 +8296,7 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>À générer</t>
+          <t>Généré le 28/09 (Soul V2)</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
@@ -8280,7 +8304,11 @@
           <t>Corbeille de fruits de fêtes en kraft avec ruban</t>
         </is>
       </c>
-      <c r="E63" s="2" t="inlineStr"/>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>017b0ad6</t>
+        </is>
+      </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
           <t>généré</t>
@@ -8380,7 +8408,7 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>À générer</t>
+          <t>Généré le 28/09 (Soul V2)</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -8388,7 +8416,11 @@
           <t>Food-truck sur une place de marché à midi</t>
         </is>
       </c>
-      <c r="E66" s="2" t="inlineStr"/>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>b2cab08c</t>
+        </is>
+      </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
           <t>généré</t>
@@ -8470,7 +8502,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Image Soul V2 (≈0,12 cr) ; si le rendu déçoit, Nano Banana 2 (≈2 cr). Animer en zoom lent dans CapCut.</t>
+          <t>✓ Généré le 28/09 avec Soul V2 (0,12 cr), ID bc0a40ea. Animer en zoom lent dans CapCut ; si le rendu déçoit, regénérer avec Nano Banana 2 (≈2 cr).</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -8480,7 +8512,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>0,12 à 2</t>
+          <t>0,12 (payé)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -8502,7 +8534,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Image Soul V2 (≈0,12 cr) ; si le rendu déçoit, Nano Banana 2 (≈2 cr). Animer en zoom lent dans CapCut.</t>
+          <t>✓ Généré le 28/09 avec Soul V2 (0,12 cr), ID f8b0e3e7. Animer en zoom lent dans CapCut ; si le rendu déçoit, regénérer avec Nano Banana 2 (≈2 cr).</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -8512,7 +8544,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>0,12 à 2</t>
+          <t>0,12 (payé)</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -8534,7 +8566,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Image Soul V2 (≈0,12 cr) ; si le rendu déçoit, Nano Banana 2 (≈2 cr). Animer en zoom lent dans CapCut.</t>
+          <t>✓ Généré le 28/09 avec Soul V2 (0,12 cr), ID c0a50f0f. Animer en zoom lent dans CapCut ; si le rendu déçoit, regénérer avec Nano Banana 2 (≈2 cr).</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -8544,7 +8576,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>0,12 à 2</t>
+          <t>0,12 (payé)</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -8566,7 +8598,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Image Soul V2 (≈0,12 cr) ; si le rendu déçoit, Nano Banana 2 (≈2 cr). Animer en zoom lent dans CapCut.</t>
+          <t>✓ Généré le 28/09 avec Soul V2 (0,12 cr), ID aa97dfff. Animer en zoom lent dans CapCut ; si le rendu déçoit, regénérer avec Nano Banana 2 (≈2 cr).</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -8576,7 +8608,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>0,12 à 2</t>
+          <t>0,12 (payé)</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -8598,7 +8630,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Image Soul V2 (≈0,12 cr) ; si le rendu déçoit, Nano Banana 2 (≈2 cr). Animer en zoom lent dans CapCut.</t>
+          <t>✓ Généré le 28/09 avec Soul V2 (0,12 cr), ID 57b69978. Animer en zoom lent dans CapCut ; si le rendu déçoit, regénérer avec Nano Banana 2 (≈2 cr).</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -8608,7 +8640,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>0,12 à 2</t>
+          <t>0,12 (payé)</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -8630,7 +8662,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Image Soul V2 (≈0,12 cr) ; si le rendu déçoit, Nano Banana 2 (≈2 cr). Animer en zoom lent dans CapCut.</t>
+          <t>✓ Généré le 28/09 avec Soul V2 (0,12 cr), ID b2cab08c. Animer en zoom lent dans CapCut ; si le rendu déçoit, regénérer avec Nano Banana 2 (≈2 cr).</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -8640,7 +8672,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>0,12 à 2</t>
+          <t>0,12 (payé)</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -8662,7 +8694,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Image Soul V2 (≈0,12 cr) ; si le rendu déçoit, Nano Banana 2 (≈2 cr). Animer en zoom lent dans CapCut.</t>
+          <t>✓ Généré le 28/09 avec Soul V2 (0,12 cr), ID dab06dad. Animer en zoom lent dans CapCut ; si le rendu déçoit, regénérer avec Nano Banana 2 (≈2 cr).</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -8672,7 +8704,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>0,12 à 2</t>
+          <t>0,12 (payé)</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -8694,7 +8726,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Image Soul V2 (≈0,12 cr) ; si le rendu déçoit, Nano Banana 2 (≈2 cr). Animer en zoom lent dans CapCut.</t>
+          <t>✓ Généré le 28/09 avec Soul V2 (0,12 cr), ID 017b0ad6. Animer en zoom lent dans CapCut ; si le rendu déçoit, regénérer avec Nano Banana 2 (≈2 cr).</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -8704,7 +8736,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>0,12 à 2</t>
+          <t>0,12 (payé)</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">

</xml_diff>

<commit_message>
docs: plan de génération vidéo 1080p pour novembre
13 plans Seedance à générer à réception des crédits (8 à partir des images
Soul, 6 nouveaux), priorisés par nombre de posts qui les utilisent.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FMRjbXSp29HtAam2YYiN3d
</commit_message>
<xml_diff>
--- a/docs/dossier-production-novembre-2026.xlsx
+++ b/docs/dossier-production-novembre-2026.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Calendrier optimisé" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Bibliothèque de plans" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="À produire" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Vidéos à générer (J+2)" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Calendrier optimisé'!$A$1:$S$57</definedName>
@@ -624,11 +625,11 @@
       <c r="M2" s="2" t="inlineStr">
         <is>
           <t>1. [NW-VITRINE-NOEL] « J-51 » en énorme · VO : Il reste cinquante et un jours. Et tes clients de Noël ont déjà commencé à chercher.
-2. [GE-RUSH] L'an dernier, le 23, c'était ça.
+2. [V-FILE-24] L'an dernier, le 23, c'était ça.
 3. [PR-CARNET] Des commandes partout. Et deux oubliées.
 4. [SCR09] Cette année : ton catalogue de fêtes en ligne, avec une date limite.
 5. [BO-EMBALLE] Chaque commande est réglée ou garantie.
-6. [PR-SAC-ATTEND] Le 24, les sacs attendent leur client.
+6. [V-SAC-NOEL] Le 24, les sacs attendent leur client.
 7. [NW-VITRINE-NOEL] Tu ouvres quand ? Écris NOËL. (silence 1,5 s)</t>
         </is>
       </c>
@@ -654,7 +655,7 @@
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>NW-VITRINE-NOEL, SCR09</t>
+          <t>NW-VITRINE-NOEL, SCR09, V-FILE-24, V-SAC-NOEL</t>
         </is>
       </c>
       <c r="S2" s="2" t="inlineStr">
@@ -1018,10 +1019,11 @@
         <is>
           <t>1. [NW-FRUITSMER] « 31/12 · 10 h » · VO : Le trente et un à dix heures, il y a quarante plateaux à sortir.
 2. [PO-ETAL] Et pas un seul dans le carnet.
-3. [SCR09] Ils ont été commandés en ligne. Réglés d'avance.
-4. [SCR04] Chacun a son créneau. Dix minutes, pas plus.
-5. [PO-EMBALLE] Tu emballes à l'heure. Sur glace jusqu'au retrait.
-6. [NW-FRUITSMER] Tes plateaux du 31, tu les prends jusqu'à quand ?</t>
+3. [V-TEL-NUIT] Ils ont été commandés en ligne, souvent le soir.
+4. [SCR09] Réglés d'avance.
+5. [SCR04] Chacun a son créneau. Dix minutes, pas plus.
+6. [PO-EMBALLE] Tu emballes à l'heure. Sur glace jusqu'au retrait.
+7. [NW-FRUITSMER] Tes plateaux du 31, tu les prends jusqu'à quand ?</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -1046,7 +1048,7 @@
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>NW-FRUITSMER, SCR04, SCR09</t>
+          <t>NW-FRUITSMER, SCR04, SCR09, V-TEL-NUIT</t>
         </is>
       </c>
       <c r="S6" s="2" t="inlineStr">
@@ -1503,7 +1505,7 @@
 3. [MD] Slide 3 : bouton Facebook « Commander »
 4. [OCT-CARROUSELS] Slide 4 : fiche Google (reprendre une slide de C06)
 5. [SCR07] Slide 5 : SMS aux habitués
-6. [NW-VITRINE-NOEL] Slide 6 : QR code en vitrine
+6. [V-QR-SCAN] Slide 6 : QR code en vitrine (image extraite)
 7. [MD] Slide 7 : checklist</t>
         </is>
       </c>
@@ -1529,7 +1531,7 @@
       </c>
       <c r="R11" s="2" t="inlineStr">
         <is>
-          <t>NW-VITRINE-NOEL, SCR07</t>
+          <t>SCR07, V-QR-SCAN</t>
         </is>
       </c>
       <c r="S11" s="2" t="inlineStr">
@@ -1781,7 +1783,7 @@
         <is>
           <t>1. [PZ-FOUR] « 12 € » · VO : Cette pizza à douze euros, il t'en reste combien ?
 2. [MD] Une part s'envole : « −3,60 € »
-3. [MD] Soixante pizzas ce soir : « −216 € »
+3. [V-PIZZA-RUSH] Soixante pizzas ce soir : compteur « −216 € » en surimpression
 4. [SCR02] Sur ta propre boutique : zéro pour cent.
 5. [PZ-TABLE] Et le client, c'est le tien.
 6. [PZ-FOUR] Ta plateforme te prend combien ? Le pourcentage suffit.</t>
@@ -1809,7 +1811,7 @@
       </c>
       <c r="R14" s="2" t="inlineStr">
         <is>
-          <t>SCR02</t>
+          <t>SCR02, V-PIZZA-RUSH</t>
         </is>
       </c>
       <c r="S14" s="2" t="inlineStr">
@@ -1972,9 +1974,10 @@
         <is>
           <t>1. [GE-SAC-GLISSE] VO : Ce sac part avec une plateforme. Et il revient chez toi.
 2. [IM-MAINS-TEL] Dedans, une carte : « la prochaine fois, commande directement ».
-3. [SCR02] Le client scanne. Il commande chez toi.
-4. [PZ-TABLE] Sans commission. Et il revient.
-5. [MD] Tu mets une carte dans tes sacs ? Oui ou non.</t>
+3. [V-QR-SCAN] Le client scanne.
+4. [SCR02] Il commande chez toi.
+5. [PZ-TABLE] Sans commission. Et il revient.
+6. [MD] Tu mets une carte dans tes sacs ? Oui ou non.</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
@@ -1999,7 +2002,7 @@
       </c>
       <c r="R16" s="2" t="inlineStr">
         <is>
-          <t>SCR02</t>
+          <t>SCR02, V-QR-SCAN</t>
         </is>
       </c>
       <c r="S16" s="2" t="inlineStr">
@@ -3087,7 +3090,7 @@
 2. [GE-RIDEAU-SOIR] Le rideau descend. Personne n'est venu.
 3. [SCR05] Cette année, la carte est enregistrée. Pas débitée : une garantie.
 4. [MD] C'est toi qui choisis le pourcentage retenu.
-5. [GE-SAC-GLISSE] Et les clients viennent.
+5. [V-REMISE-NOEL] Et les clients viennent.
 6. [NW-BUCHE] Un no-show à Noël, ça doit se payer ? Oui ou non.</t>
         </is>
       </c>
@@ -3113,7 +3116,7 @@
       </c>
       <c r="R28" s="2" t="inlineStr">
         <is>
-          <t>NW-BUCHE, SCR05</t>
+          <t>NW-BUCHE, SCR05, V-REMISE-NOEL</t>
         </is>
       </c>
       <c r="S28" s="2" t="inlineStr">
@@ -3468,7 +3471,8 @@
 3. [SCR03] Le prix. La date limite.
 4. [NW-BUCHE] La bûche.
 5. [NW-FRUITSMER] Le plateau.
-6. [MD] Chrono arrêté · Tu commences quand ?</t>
+6. [V-TEL-NUIT] Et les commandes arrivent.
+7. [MD] Chrono arrêté · Tu commences quand ?</t>
         </is>
       </c>
       <c r="N32" s="2" t="inlineStr">
@@ -3493,7 +3497,7 @@
       </c>
       <c r="R32" s="2" t="inlineStr">
         <is>
-          <t>NW-BUCHE, NW-FRUITSMER, NW-VOLAILLE, SCR03</t>
+          <t>NW-BUCHE, NW-FRUITSMER, NW-VOLAILLE, SCR03, V-TEL-NUIT</t>
         </is>
       </c>
       <c r="S32" s="2" t="inlineStr">
@@ -4396,11 +4400,12 @@
       <c r="M42" s="2" t="inlineStr">
         <is>
           <t>1. [NW-VITRINE-NOEL] « J-31 » · VO : Trente et un jours. Et une semaine pour tout ouvrir.
-2. [GE-RUSH] Sinon, le 23 ressemblera à celui de l'an dernier.
+2. [V-FILE-24] Sinon, le 23 ressemblera à celui de l'an dernier.
 3. [SCR09] Catalogue de fêtes, date limite.
 4. [SCR04] Créneaux du 22 au 24.
 5. [SCR05] Empreinte ou acompte.
-6. [NW-VITRINE-NOEL] Tu ouvres quand ? Écris NOËL.</t>
+6. [V-SAC-NOEL] Et le 24, tout est prêt.
+7. [NW-VITRINE-NOEL] Tu ouvres quand ? Écris NOËL.</t>
         </is>
       </c>
       <c r="N42" s="2" t="inlineStr">
@@ -4425,7 +4430,7 @@
       </c>
       <c r="R42" s="2" t="inlineStr">
         <is>
-          <t>NW-VITRINE-NOEL, SCR04, SCR05, SCR09</t>
+          <t>NW-VITRINE-NOEL, SCR04, SCR05, SCR09, V-FILE-24, V-SAC-NOEL</t>
         </is>
       </c>
       <c r="S42" s="2" t="inlineStr">
@@ -4589,11 +4594,11 @@
       </c>
       <c r="M44" s="2" t="inlineStr">
         <is>
-          <t>1. [BL-FOUR] VO : Le 24 au matin, ta file va jusqu'au trottoir. Sauf si…
+          <t>1. [V-FILE-24] VO : Le 24 au matin, ta file va jusqu'au trottoir. Sauf si…
 2. [NW-BUCHE] …tes bûches se commandent jusqu'au 20.
 3. [SCR04] Retraits étalés : le 22, le 23, le 24.
 4. [BL-SAC] Chaque client a son heure.
-5. [GE-SAC-GLISSE] Dix secondes au comptoir.
+5. [V-REMISE-NOEL] Dix secondes au comptoir.
 6. [BL-FOUR] Tes bûches, date limite quand ?</t>
         </is>
       </c>
@@ -4619,7 +4624,7 @@
       </c>
       <c r="R44" s="2" t="inlineStr">
         <is>
-          <t>NW-BUCHE, SCR04</t>
+          <t>NW-BUCHE, SCR04, V-FILE-24, V-REMISE-NOEL</t>
         </is>
       </c>
       <c r="S44" s="2" t="inlineStr">
@@ -4780,7 +4785,8 @@
 2. [SCR01] Trente secondes pour la démo.
 3. [SCR03] Tes produits de fêtes.
 4. [SCR04] Tes créneaux.
-5. [NW-VITRINE-NOEL] Tu la crées quand ? Écris DEMO.</t>
+5. [V-TEL-NUIT] Et les commandes arrivent, même la nuit.
+6. [NW-VITRINE-NOEL] Tu la crées quand ? Écris DEMO.</t>
         </is>
       </c>
       <c r="N46" s="2" t="inlineStr">
@@ -4805,7 +4811,7 @@
       </c>
       <c r="R46" s="2" t="inlineStr">
         <is>
-          <t>NW-VITRINE-NOEL, SCR01, SCR03, SCR04</t>
+          <t>NW-VITRINE-NOEL, SCR01, SCR03, SCR04, V-TEL-NUIT</t>
         </is>
       </c>
       <c r="S46" s="2" t="inlineStr">
@@ -4869,7 +4875,7 @@
       <c r="L47" s="2" t="inlineStr"/>
       <c r="M47" s="2" t="inlineStr">
         <is>
-          <t>1. [NW-VITRINE-NOEL] Slide 1 : vitrine avec un vrai QR incrusté sur le sticker vierge
+          <t>1. [V-QR-SCAN] Slide 1 : image extraite, vrai QR incrusté sur le sticker vierge
 2. [MD] Slides 2 à 5 : emplacement, texte, annonce
 3. [MD] Slide 6 : récap</t>
         </is>
@@ -4896,7 +4902,7 @@
       </c>
       <c r="R47" s="2" t="inlineStr">
         <is>
-          <t>NW-VITRINE-NOEL</t>
+          <t>V-QR-SCAN</t>
         </is>
       </c>
       <c r="S47" s="2" t="inlineStr">
@@ -4964,7 +4970,7 @@
       </c>
       <c r="M48" s="2" t="inlineStr">
         <is>
-          <t>1. [PZ-FOUR] VO : Vingt heures. Trente commandes en même temps. Le four ne suit pas.
+          <t>1. [V-PIZZA-RUSH] VO : Vingt heures. Trente commandes en même temps. Le four ne suit pas.
 2. [MD] Graphique : un pic → un plateau
 3. [SCR04] Quinze minutes par créneau. Huit pizzas maximum.
 4. [PZ-TABLE] La salle respire.
@@ -4994,7 +5000,7 @@
       </c>
       <c r="R48" s="2" t="inlineStr">
         <is>
-          <t>NW-SALLE-6, SCR04</t>
+          <t>NW-SALLE-6, SCR04, V-PIZZA-RUSH</t>
         </is>
       </c>
       <c r="S48" s="2" t="inlineStr">
@@ -5342,10 +5348,10 @@
       <c r="M52" s="2" t="inlineStr">
         <is>
           <t>1. [PR-CARNET2] « Erreur n°1 » · VO : Erreur numéro un : pas de date limite.
-2. [GE-RUSH] Numéro deux : tous les retraits le 24.
+2. [V-FILE-24] Numéro deux : tous les retraits le 24.
 3. [GE-PORTE-MOT] Numéro trois : aucun acompte. Et personne ne vient.
 4. [SCR09] La correction : date limite, créneaux, empreinte.
-5. [PR-SAC-ATTEND] Et ton 24 est presque calme.
+5. [V-SAC-NOEL] Et ton 24 est presque calme.
 6. [MD] Laquelle tu fais ? 1, 2 ou 3 ?</t>
         </is>
       </c>
@@ -5371,7 +5377,7 @@
       </c>
       <c r="R52" s="2" t="inlineStr">
         <is>
-          <t>SCR09</t>
+          <t>SCR09, V-FILE-24, V-SAC-NOEL</t>
         </is>
       </c>
       <c r="S52" s="2" t="inlineStr">
@@ -5723,7 +5729,7 @@
 2. [SCR09] Un : tes précommandes sont ouvertes.
 3. [SCR04] Deux : tes retraits sont étalés.
 4. [SCR07] Trois : tes clients sont prévenus.
-5. [PR-REMISE] Et le 24, tu remets des sacs.
+5. [V-REMISE-NOEL] Et le 24, tu remets des paquets.
 6. [NW-VITRINE-NOEL] Tu es prêt ? Écris DEMO.</t>
         </is>
       </c>
@@ -5749,7 +5755,7 @@
       </c>
       <c r="R56" s="2" t="inlineStr">
         <is>
-          <t>NW-VITRINE-NOEL, SCR04, SCR07, SCR09</t>
+          <t>NW-VITRINE-NOEL, SCR04, SCR07, SCR09, V-REMISE-NOEL</t>
         </is>
       </c>
       <c r="S56" s="2" t="inlineStr">
@@ -5864,7 +5870,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H66"/>
+  <dimension ref="A1:H72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5951,11 +5957,11 @@
         </is>
       </c>
       <c r="G2" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>8, 9, 15, 17, 27, 43</t>
+          <t>8, 9, 15, 17</t>
         </is>
       </c>
     </row>
@@ -6002,7 +6008,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>PR-REMISE</t>
+          <t>GE-NOTIF</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -6017,12 +6023,12 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>POV : le primeur tend le sac par-dessus le comptoir</t>
+          <t>Smartphone posé sur le comptoir, l'écran s'allume (notification)</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>0f83850c</t>
+          <t>574f5ccc</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -6035,14 +6041,14 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>21, 23, 55</t>
+          <t>17, 23, 37</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>GE-RUSH</t>
+          <t>PZ-FOUR</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -6057,12 +6063,12 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Rush en boulangerie : combiné + bloc + papiers partout</t>
+          <t>Pizza sortie du four à bois</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>126bdc8f</t>
+          <t>1ba5f18d</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -6075,19 +6081,19 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>1, 41, 51</t>
+          <t>13, 19, 47</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>GE-NOTIF</t>
+          <t>IM-MAINS-TEL</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Vidéo 5 s</t>
+          <t>Image 9:16</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -6097,12 +6103,12 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Smartphone posé sur le comptoir, l'écran s'allume (notification)</t>
+          <t>Deux mains se passent un smartphone par-dessus le comptoir</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>574f5ccc</t>
+          <t>fb073ff8</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -6115,34 +6121,34 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>17, 23, 37</t>
+          <t>12, 15, 26</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>PZ-FOUR</t>
+          <t>OCT-CARROUSELS</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Vidéo 5 s</t>
+          <t>30 carrousels</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Highfield</t>
+          <t>Drive « carrousels »</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Pizza sortie du four à bois</t>
+          <t>C01 à C30 en 1080×1350 : gabarits à dupliquer (même charte)</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>1ba5f18d</t>
+          <t>dossier</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -6155,19 +6161,19 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>13, 19, 47</t>
+          <t>2, 10, 14</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>IM-MAINS-TEL</t>
+          <t>PR-REMISE</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Image 9:16</t>
+          <t>Vidéo 5 s</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -6177,12 +6183,12 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Deux mains se passent un smartphone par-dessus le comptoir</t>
+          <t>POV : le primeur tend le sac par-dessus le comptoir</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>fb073ff8</t>
+          <t>0f83850c</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -6191,38 +6197,38 @@
         </is>
       </c>
       <c r="G8" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>12, 15, 26</t>
+          <t>21, 23</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>OCT-CARROUSELS</t>
+          <t>PR-CARNET</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>30 carrousels</t>
+          <t>Vidéo 5 s</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Drive « carrousels »</t>
+          <t>Highfield</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>C01 à C30 en 1080×1350 : gabarits à dupliquer (même charte)</t>
+          <t>Carnet de commandes surchargé montré à la caméra</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>dossier</t>
+          <t>1d2b382b</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -6231,18 +6237,18 @@
         </is>
       </c>
       <c r="G9" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>2, 10, 14</t>
+          <t>1, 7</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>PR-SAC-ATTEND</t>
+          <t>PR-PESEE</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -6257,12 +6263,12 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Sac kraft (artichauts) seul sur le comptoir, personne</t>
+          <t>Mains qui pèsent des tomates, téléphone au fond qui devient net</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>de24487c</t>
+          <t>17745e43</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -6275,14 +6281,14 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>1, 51</t>
+          <t>8, 33</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>PR-CARNET</t>
+          <t>BL-FOUR</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -6297,12 +6303,12 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Carnet de commandes surchargé montré à la caméra</t>
+          <t>Boulanger qui enfourne des baguettes à l'aube</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>1d2b382b</t>
+          <t>1790adeb</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -6315,14 +6321,14 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>1, 7</t>
+          <t>24, 43</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>PR-PESEE</t>
+          <t>BO-EMBALLE</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -6337,12 +6343,12 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Mains qui pèsent des tomates, téléphone au fond qui devient net</t>
+          <t>Boucher qui emballe un rôti, 3 paquets identiques</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>17745e43</t>
+          <t>1e6191a0</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -6355,14 +6361,14 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>8, 33</t>
+          <t>1, 33</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>BL-FOUR</t>
+          <t>FR-PLATEAU</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -6377,12 +6383,12 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Boulanger qui enfourne des baguettes à l'aube</t>
+          <t>Fromager qui compose un plateau sur planche en bois</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>1790adeb</t>
+          <t>fda2d387</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -6395,14 +6401,14 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>24, 43</t>
+          <t>8, 42</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>BO-EMBALLE</t>
+          <t>FL-DEVANTURE</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -6417,12 +6423,12 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Boucher qui emballe un rôti, 3 paquets identiques</t>
+          <t>Devanture de fleuriste au petit matin, seaux de fleurs</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>1e6191a0</t>
+          <t>da001057</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -6435,14 +6441,14 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>1, 33</t>
+          <t>9, 49</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>FR-PLATEAU</t>
+          <t>FL-BOUQUET</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -6457,12 +6463,12 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Fromager qui compose un plateau sur planche en bois</t>
+          <t>Fleuriste qui emballe un bouquet dans du kraft</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>fda2d387</t>
+          <t>60ce7b44</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -6475,14 +6481,14 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>8, 42</t>
+          <t>9, 49</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>FL-DEVANTURE</t>
+          <t>PO-ETAL</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -6497,12 +6503,12 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Devanture de fleuriste au petit matin, seaux de fleurs</t>
+          <t>Travelling sur l'étal de poissons sur glace</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>da001057</t>
+          <t>9e0e4cdf</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -6515,14 +6521,14 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>9, 49</t>
+          <t>5, 37</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>FL-BOUQUET</t>
+          <t>PO-EMBALLE</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -6537,12 +6543,12 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Fleuriste qui emballe un bouquet dans du kraft</t>
+          <t>Poissonnier qui emballe un filet dans du papier</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>60ce7b44</t>
+          <t>d0c8f10c</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -6555,19 +6561,19 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>9, 49</t>
+          <t>5, 37</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>PO-ETAL</t>
+          <t>IM-TEL-NOIR</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Vidéo 5 s</t>
+          <t>Image 9:16</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -6577,12 +6583,12 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Travelling sur l'étal de poissons sur glace</t>
+          <t>Smartphone écran noir sur comptoir, artichauts : support pour incruster une capture d'écran</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>9e0e4cdf</t>
+          <t>26c0d73e</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -6595,14 +6601,14 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>5, 37</t>
+          <t>10, 34</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>PO-EMBALLE</t>
+          <t>PR-RIDEAU</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -6617,12 +6623,12 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Poissonnier qui emballe un filet dans du papier</t>
+          <t>Primeur : le rideau se lève à l'aube, vue de l'intérieur vers la rue</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>d0c8f10c</t>
+          <t>788b7105</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -6631,23 +6637,23 @@
         </is>
       </c>
       <c r="G19" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>5, 37</t>
+          <t>21</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>IM-TEL-NOIR</t>
+          <t>PR-REMPLIT</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Image 9:16</t>
+          <t>Vidéo 5 s</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -6657,12 +6663,12 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Smartphone écran noir sur comptoir, artichauts : support pour incruster une capture d'écran</t>
+          <t>Mains qui remplissent un sac kraft (artichauts, aubergine, avocats)</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>26c0d73e</t>
+          <t>1e6b8870</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -6671,18 +6677,18 @@
         </is>
       </c>
       <c r="G20" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>10, 34</t>
+          <t>21</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>PR-RIDEAU</t>
+          <t>PR-CARNET2</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -6697,12 +6703,12 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Primeur : le rideau se lève à l'aube, vue de l'intérieur vers la rue</t>
+          <t>Carnet taché, gribouillé, pages cornées</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>788b7105</t>
+          <t>56224443</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -6715,14 +6721,14 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>51</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>PR-REMPLIT</t>
+          <t>PR-LISTE</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -6737,12 +6743,12 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Mains qui remplissent un sac kraft (artichauts, aubergine, avocats)</t>
+          <t>Crayon qui hésite sur une liste puis coche une ligne</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>1e6b8870</t>
+          <t>3af5268c</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -6762,7 +6768,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>PR-CARNET2</t>
+          <t>CL-CANAPE</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -6777,12 +6783,12 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Carnet taché, gribouillé, pages cornées</t>
+          <t>Salon le soir, cliente sur le canapé avec son téléphone</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>56224443</t>
+          <t>868a50a0</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -6795,14 +6801,14 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>23</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>PR-LISTE</t>
+          <t>GE-RACCROCHE</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -6817,12 +6823,12 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Crayon qui hésite sur une liste puis coche une ligne</t>
+          <t>Main qui raccroche un téléphone mural</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>3af5268c</t>
+          <t>aac7bebc</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -6835,14 +6841,14 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>7</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>CL-CANAPE</t>
+          <t>GE-PORTE-MOT</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -6857,12 +6863,12 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Salon le soir, cliente sur le canapé avec son téléphone</t>
+          <t>Porte fermée sous la pluie, mot scotché sur la vitre</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>868a50a0</t>
+          <t>02bf3e32</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -6875,14 +6881,14 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>51</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>GE-RACCROCHE</t>
+          <t>GE-RIDEAU-SOIR</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -6897,12 +6903,12 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Main qui raccroche un téléphone mural</t>
+          <t>Rideau métallique baissé au crépuscule</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>aac7bebc</t>
+          <t>9ac967f2</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -6915,14 +6921,14 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>27</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>GE-PORTE-MOT</t>
+          <t>BL-SAC</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -6937,12 +6943,12 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Porte fermée sous la pluie, mot scotché sur la vitre</t>
+          <t>Baguettes et boule glissées dans un sac kraft</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>02bf3e32</t>
+          <t>467bec5c</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -6955,14 +6961,14 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>43</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>GE-RIDEAU-SOIR</t>
+          <t>BO-FICELLE</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -6977,12 +6983,12 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Rideau métallique baissé au crépuscule</t>
+          <t>Boucher qui ficelle un rôti</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>9ac967f2</t>
+          <t>2080181b</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -6995,14 +7001,14 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>33</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>BL-SAC</t>
+          <t>TR-CANAPES</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -7017,12 +7023,12 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Baguettes et boule glissées dans un sac kraft</t>
+          <t>Traiteur qui finit un plateau de canapés de fête</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>467bec5c</t>
+          <t>ea82cc27</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -7035,14 +7041,14 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>6</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>BO-FICELLE</t>
+          <t>TR-COUVERCLE</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -7057,12 +7063,12 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Boucher qui ficelle un rôti</t>
+          <t>Traiteur qui ferme un plateau, 3 plateaux identiques</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>2080181b</t>
+          <t>2cb32eed</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -7075,19 +7081,19 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>35</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>TR-CANAPES</t>
+          <t>UGC-TR-1</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Vidéo 5 s</t>
+          <t>Vidéo 15 s</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -7097,12 +7103,12 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Traiteur qui finit un plateau de canapés de fête</t>
+          <t>Traiteur face caméra (muet) : la grosse commande jamais récupérée</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>ea82cc27</t>
+          <t>ee6ae008</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -7115,19 +7121,19 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>35</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>TR-COUVERCLE</t>
+          <t>UGC-TR-2</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Vidéo 5 s</t>
+          <t>Vidéo 15 s</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -7137,12 +7143,12 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Traiteur qui ferme un plateau, 3 plateaux identiques</t>
+          <t>Traiteur (muet) : aucun recours… sauf une carte, comme à l'hôtel</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>2cb32eed</t>
+          <t>c985ea20</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -7162,7 +7168,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>UGC-TR-1</t>
+          <t>UGC-TR-3</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -7177,12 +7183,12 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Traiteur face caméra (muet) : la grosse commande jamais récupérée</t>
+          <t>Traiteur (muet) : montre son téléphone, pose la question au spectateur</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>ee6ae008</t>
+          <t>5e737f10</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -7202,12 +7208,12 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>UGC-TR-2</t>
+          <t>IM-MATERIEL</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Vidéo 15 s</t>
+          <t>4 images</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -7217,12 +7223,12 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Traiteur (muet) : aucun recours… sauf une carte, comme à l'hôtel</t>
+          <t>Terminal CB, caisse, tablette, imprimante à tickets (fond gris)</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>c985ea20</t>
+          <t>653f5d81…</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -7235,19 +7241,19 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>20</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>UGC-TR-3</t>
+          <t>IM-ETAL-OR</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Vidéo 15 s</t>
+          <t>Image 9:16</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -7257,12 +7263,12 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Traiteur (muet) : montre son téléphone, pose la question au spectateur</t>
+          <t>Étal de primeur au soleil couchant, zone vide pour le texte</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>5e737f10</t>
+          <t>a01ffb0b</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -7275,19 +7281,19 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>39</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>IM-MATERIEL</t>
+          <t>PR-SAC-ATTEND</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>4 images</t>
+          <t>Vidéo 5 s</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -7297,12 +7303,12 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Terminal CB, caisse, tablette, imprimante à tickets (fond gris)</t>
+          <t>Sac kraft (artichauts) seul sur le comptoir, personne</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>653f5d81…</t>
+          <t>de24487c</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -7311,23 +7317,19 @@
         </is>
       </c>
       <c r="G36" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H36" s="2" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="H36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>IM-ETAL-OR</t>
+          <t>PR-RUE</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Image 9:16</t>
+          <t>Vidéo 5 s</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -7337,12 +7339,12 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Étal de primeur au soleil couchant, zone vide pour le texte</t>
+          <t>POV marche sous la pluie dans une rue normande jusqu'au primeur</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>a01ffb0b</t>
+          <t>2aa815cf</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -7351,18 +7353,14 @@
         </is>
       </c>
       <c r="G37" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H37" s="2" t="inlineStr">
-        <is>
-          <t>39</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="H37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>PR-RUE</t>
+          <t>PR-DEVANTURE</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -7377,12 +7375,12 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>POV marche sous la pluie dans une rue normande jusqu'au primeur</t>
+          <t>Push-in lent sur la devanture du primeur au petit matin</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>2aa815cf</t>
+          <t>0f8b56ca</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -7398,7 +7396,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>PR-DEVANTURE</t>
+          <t>CL-SENIOR</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -7413,12 +7411,12 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Push-in lent sur la devanture du primeur au petit matin</t>
+          <t>Mains âgées qui tapent sur un smartphone, tasse de thé</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>0f8b56ca</t>
+          <t>409f3c0e</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -7434,7 +7432,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>CL-SENIOR</t>
+          <t>GE-BLOC</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -7449,12 +7447,12 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Mains âgées qui tapent sur un smartphone, tasse de thé</t>
+          <t>Main qui note une commande sur un bloc</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>409f3c0e</t>
+          <t>d6d1eb4c</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -7470,7 +7468,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>GE-BLOC</t>
+          <t>GE-RUSH</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -7485,12 +7483,12 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Main qui note une commande sur un bloc</t>
+          <t>Rush en boulangerie : combiné + bloc + papiers partout</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>d6d1eb4c</t>
+          <t>126bdc8f</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -7722,47 +7720,43 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>NW-VITRINE-NOEL</t>
+          <t>SCR02</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Image 9:16 → zoom</t>
+          <t>Capture écran</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Généré le 28/09 (Soul V2)</t>
+          <t>À filmer (gratuit)</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Devanture de commerce le soir, décorée pour Noël, sticker vierge sur la vitre</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>bc0a40ea</t>
-        </is>
-      </c>
+          <t>Parcours client sur mobile : produit → créneau → paiement → confirmation</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr"/>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>généré</t>
+          <t>à filmer</t>
         </is>
       </c>
       <c r="G48" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>1, 10, 41, 45, 46, 50, 53, 55</t>
+          <t>9, 13, 15, 17, 19, 23, 37</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>SCR02</t>
+          <t>SCR05</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -7777,7 +7771,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Parcours client sur mobile : produit → créneau → paiement → confirmation</t>
+          <t>Activer l'empreinte bancaire (%) + ce que voit le client</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr"/>
@@ -7787,39 +7781,43 @@
         </is>
       </c>
       <c r="G49" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>9, 13, 15, 17, 19, 23, 37</t>
+          <t>2, 27, 28, 29, 35, 41</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>SCR05</t>
+          <t>NW-VITRINE-NOEL</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Capture écran</t>
+          <t>Image 9:16 → zoom</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>À filmer (gratuit)</t>
+          <t>Généré le 28/09 (Soul V2)</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Activer l'empreinte bancaire (%) + ce que voit le client</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr"/>
+          <t>Devanture de commerce le soir, décorée pour Noël, sticker vierge sur la vitre</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>bc0a40ea</t>
+        </is>
+      </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>à filmer</t>
+          <t>généré</t>
         </is>
       </c>
       <c r="G50" s="2" t="n">
@@ -7827,7 +7825,7 @@
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>2, 27, 28, 29, 35, 41</t>
+          <t>1, 41, 45, 50, 53, 55</t>
         </is>
       </c>
     </row>
@@ -7910,43 +7908,43 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>SCR01</t>
+          <t>V-FILE-24</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Capture écran</t>
+          <t>Vidéo 5 s 1080p</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>À filmer (gratuit)</t>
+          <t>Vidéo à générer (crédits J+2)</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Création d'une démo en continu, chrono visible : métier → nom → aperçu</t>
+          <t>Nouveau · File d'attente jusqu'au trottoir devant une boulangerie, matin du 24</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr"/>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>à filmer</t>
+          <t>vidéo</t>
         </is>
       </c>
       <c r="G53" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>3, 19, 45</t>
+          <t>1, 41, 43, 51</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>SCR06</t>
+          <t>SCR01</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -7961,7 +7959,7 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Produit au kilo : choix du poids + ajustement à la pesée</t>
+          <t>Création d'une démo en continu, chrono visible : métier → nom → aperçu</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr"/>
@@ -7975,14 +7973,14 @@
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>4, 8, 33</t>
+          <t>3, 19, 45</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>SCR07</t>
+          <t>SCR06</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -7997,7 +7995,7 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>SMS « commande prête » reçu sur un vrai téléphone</t>
+          <t>Produit au kilo : choix du poids + ajustement à la pesée</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr"/>
@@ -8011,14 +8009,14 @@
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>10, 33, 55</t>
+          <t>4, 8, 33</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>SCR08</t>
+          <t>SCR07</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -8033,7 +8031,7 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Livraison : zone, minimum, frais, créneaux</t>
+          <t>SMS « commande prête » reçu sur un vrai téléphone</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr"/>
@@ -8043,195 +8041,183 @@
         </is>
       </c>
       <c r="G56" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>38, 49</t>
+          <t>10, 33, 55</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>SCR12</t>
+          <t>V-SAC-NOEL</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Capture écran</t>
+          <t>Vidéo 5 s 1080p</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>À filmer (gratuit)</t>
+          <t>Vidéo à générer (crédits J+2)</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Tableau de bord commerçant : commandes du jour</t>
+          <t>Nouveau · Étagère de retrait pleine de sacs et paquets de fêtes nominatifs (étiquettes vierges)</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr"/>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>à filmer</t>
+          <t>vidéo</t>
         </is>
       </c>
       <c r="G57" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>7, 21</t>
+          <t>1, 41, 51</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>TRN-PAUL</t>
+          <t>V-TEL-NUIT</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Tournage</t>
+          <t>Vidéo 5 s 1080p</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>À filmer (gratuit)</t>
+          <t>Vidéo à générer (crédits J+2)</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Paul en selfie, 30 s, lumière naturelle</t>
+          <t>Nouveau · Téléphone sur le comptoir la nuit, l'écran s'allume plusieurs fois (commandes qui arrivent)</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr"/>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>à filmer</t>
+          <t>vidéo</t>
         </is>
       </c>
       <c r="G58" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>7, 36</t>
+          <t>5, 31, 45</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>NW-FRUITSMER</t>
+          <t>V-REMISE-NOEL</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Image 9:16 → zoom</t>
+          <t>Vidéo 5 s 1080p</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Généré le 28/09 (Soul V2)</t>
+          <t>Vidéo à générer (crédits J+2)</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Plateau de fruits de mer de fête sur glace, papier</t>
-        </is>
-      </c>
-      <c r="E59" s="2" t="inlineStr">
-        <is>
-          <t>c0a50f0f</t>
-        </is>
-      </c>
+          <t>Nouveau · Remise d'un paquet de fête par-dessus le comptoir, sourire implicite, rapide</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr"/>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>généré</t>
+          <t>vidéo</t>
         </is>
       </c>
       <c r="G59" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>5, 31</t>
+          <t>27, 43, 55</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>NW-VOLAILLE</t>
+          <t>V-QR-SCAN</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Image 9:16 → zoom</t>
+          <t>Vidéo 5 s 1080p</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Généré le 28/09 (Soul V2)</t>
+          <t>Vidéo à générer (crédits J+2)</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Volaille de fête ficelée sur papier boucher</t>
-        </is>
-      </c>
-      <c r="E60" s="2" t="inlineStr">
-        <is>
-          <t>aa97dfff</t>
-        </is>
-      </c>
+          <t>Nouveau · Une main scanne le sticker de la vitrine avec son téléphone</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr"/>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>généré</t>
+          <t>vidéo</t>
         </is>
       </c>
       <c r="G60" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>4, 31</t>
+          <t>10, 15, 46</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>NW-COURONNE</t>
+          <t>SCR08</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Image 9:16 → zoom</t>
+          <t>Capture écran</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Généré le 28/09 (Soul V2)</t>
+          <t>À filmer (gratuit)</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>Couronne de l'Avent sur l'établi du fleuriste</t>
-        </is>
-      </c>
-      <c r="E61" s="2" t="inlineStr">
-        <is>
-          <t>57b69978</t>
-        </is>
-      </c>
+          <t>Livraison : zone, minimum, frais, créneaux</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr"/>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>généré</t>
+          <t>à filmer</t>
         </is>
       </c>
       <c r="G61" s="2" t="n">
@@ -8239,39 +8225,35 @@
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>9, 49</t>
+          <t>38, 49</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>NW-SALLE-6</t>
+          <t>SCR12</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Image 9:16 → zoom</t>
+          <t>Capture écran</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Généré le 28/09 (Soul V2)</t>
+          <t>À filmer (gratuit)</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Salle de restaurant le soir, table de 6 dressée et vide</t>
-        </is>
-      </c>
-      <c r="E62" s="2" t="inlineStr">
-        <is>
-          <t>dab06dad</t>
-        </is>
-      </c>
+          <t>Tableau de bord commerçant : commandes du jour</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr"/>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>généré</t>
+          <t>à filmer</t>
         </is>
       </c>
       <c r="G62" s="2" t="n">
@@ -8279,39 +8261,35 @@
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>29, 47</t>
+          <t>7, 21</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>NW-PANIER-FETES</t>
+          <t>TRN-PAUL</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Image 9:16 → zoom</t>
+          <t>Tournage</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Généré le 28/09 (Soul V2)</t>
+          <t>À filmer (gratuit)</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Corbeille de fruits de fêtes en kraft avec ruban</t>
-        </is>
-      </c>
-      <c r="E63" s="2" t="inlineStr">
-        <is>
-          <t>017b0ad6</t>
-        </is>
-      </c>
+          <t>Paul en selfie, 30 s, lumière naturelle</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr"/>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>généré</t>
+          <t>à filmer</t>
         </is>
       </c>
       <c r="G63" s="2" t="n">
@@ -8319,117 +8297,353 @@
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>38, 52</t>
+          <t>7, 36</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>SCR10</t>
+          <t>NW-FRUITSMER</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Capture écran</t>
+          <t>Image 9:16 → zoom</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>À filmer (gratuit)</t>
+          <t>Généré le 28/09 (Soul V2)</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Réservation de table (boutique démo restaurant)</t>
-        </is>
-      </c>
-      <c r="E64" s="2" t="inlineStr"/>
+          <t>Plateau de fruits de mer de fête sur glace, papier</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>c0a50f0f</t>
+        </is>
+      </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>à filmer</t>
+          <t>généré</t>
         </is>
       </c>
       <c r="G64" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>5, 31</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>TRN-CLIENT</t>
+          <t>NW-VOLAILLE</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Tournage</t>
+          <t>Image 9:16 → zoom</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>À filmer (gratuit)</t>
+          <t>Généré le 28/09 (Soul V2)</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>Un vrai commerçant client, sur place, avec accord écrit</t>
-        </is>
-      </c>
-      <c r="E65" s="2" t="inlineStr"/>
+          <t>Volaille de fête ficelée sur papier boucher</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>aa97dfff</t>
+        </is>
+      </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>à filmer</t>
+          <t>généré</t>
         </is>
       </c>
       <c r="G65" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>4, 31</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
+          <t>NW-COURONNE</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Image 9:16 → zoom</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Généré le 28/09 (Soul V2)</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>Couronne de l'Avent sur l'établi du fleuriste</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>57b69978</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>généré</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>9, 49</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>NW-SALLE-6</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Image 9:16 → zoom</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Généré le 28/09 (Soul V2)</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>Salle de restaurant le soir, table de 6 dressée et vide</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>dab06dad</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>généré</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>29, 47</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>NW-PANIER-FETES</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Image 9:16 → zoom</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Généré le 28/09 (Soul V2)</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>Corbeille de fruits de fêtes en kraft avec ruban</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>017b0ad6</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>généré</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>38, 52</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>V-PIZZA-RUSH</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo 5 s 1080p</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>Vidéo à générer (crédits J+2)</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>Nouveau · Boîtes à pizza qui s'empilent au coup de feu de 20 h</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr"/>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>vidéo</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>13, 47</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>SCR10</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Capture écran</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>À filmer (gratuit)</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>Réservation de table (boutique démo restaurant)</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr"/>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>à filmer</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>TRN-CLIENT</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>Tournage</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>À filmer (gratuit)</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>Un vrai commerçant client, sur place, avec accord écrit</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr"/>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>à filmer</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
           <t>NW-FOODTRUCK</t>
         </is>
       </c>
-      <c r="B66" s="2" t="inlineStr">
+      <c r="B72" s="2" t="inlineStr">
         <is>
           <t>Image 9:16 → zoom</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr">
+      <c r="C72" s="2" t="inlineStr">
         <is>
           <t>Généré le 28/09 (Soul V2)</t>
         </is>
       </c>
-      <c r="D66" s="2" t="inlineStr">
+      <c r="D72" s="2" t="inlineStr">
         <is>
           <t>Food-truck sur une place de marché à midi</t>
         </is>
       </c>
-      <c r="E66" s="2" t="inlineStr">
+      <c r="E72" s="2" t="inlineStr">
         <is>
           <t>b2cab08c</t>
         </is>
       </c>
-      <c r="F66" s="2" t="inlineStr">
+      <c r="F72" s="2" t="inlineStr">
         <is>
           <t>généré</t>
         </is>
       </c>
-      <c r="G66" s="2" t="n">
+      <c r="G72" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H66" s="2" t="inlineStr">
+      <c r="H72" s="2" t="inlineStr">
         <is>
           <t>17</t>
         </is>
@@ -8517,7 +8731,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>1, 10, 41, 45, 46, 50, 53, 55</t>
+          <t>1, 41, 45, 50, 53, 55</t>
         </is>
       </c>
     </row>
@@ -9192,6 +9406,691 @@
           <t>2, 3, 4, 6, 10, 11, 13, 14, 15, 16, 18, 20, 24, 25, 27, 28, 30, 31, 32, 38, 39, 40, 42, 44, 46, 47, 48, 51, 52, 53, 54, 56</t>
         </is>
       </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="90" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Priorité</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Image de départ (job ID Highfield, rôle start_image)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Prompt Seedance 2.5</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Réglages</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Coût estimé</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Posts (N°)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>NW-VITRINE-NOEL</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>La vitrine de Noël s'anime : guirlande qui scintille, pluie fine, push-in très lent</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>bc0a40ea-5f0b-4131-8ed1-487546d4ad3a</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Very slow push-in toward the shop window. The warm fairy lights in the fir garland twinkle gently, fine rain falls and ripples in the puddles on the cobblestones, warm light inside the shop brightens slightly. No people appear. The blank sticker on the door stays blank. No text, no logos. Photorealistic, fine film grain. Audio: light rain, distant street, no music, no speech.</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Seedance 2.5 · 9:16 · 5 s · 1080p · audio on</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>60 crédits</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>1, 41, 45, 50, 53, 55</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>NW-BUCHE</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Mains de pâtissier qui referment la boîte de la bûche et nouent l'étiquette</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>f8b0e3e7-c783-4272-a3b3-939373237b38</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>A pastry chef's hands (navy apron, no face) enter frame, gently close the lid of the white pastry box over the log cake and tie the blank kraft label with twine, then slide the box a few centimetres forward. Soft morning window light. No text on the label, no logos. Photorealistic, fine film grain. Audio: cardboard, twine, quiet bakery, no music, no speech.</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Seedance 2.5 · 9:16 · 5 s · 1080p · audio on</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>60 crédits</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>2, 22, 27, 31, 43</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>V-FILE-24</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Nouveau · File d'attente jusqu'au trottoir devant une boulangerie, matin du 24</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>— (texte seul)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Vertical 9:16, 5 seconds, single slow lateral tracking shot on a cold winter morning in a small French town. A long queue of customers in winter coats, seen from behind and from the side at a distance (no faces), stretches out of a small bakery door along the pavement; breath visible in the cold air, Christmas garland on the shop front, warm light inside. No readable text, no logos. Photorealistic documentary, fine film grain. Audio: street murmur, cold morning, no music, no speech.</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Seedance 2.5 · 9:16 · 5 s · 1080p · audio on</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>60 crédits</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>1, 41, 43, 51</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>V-SAC-NOEL</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Nouveau · Étagère de retrait pleine de sacs et paquets de fêtes nominatifs (étiquettes vierges)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>— (texte seul)</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Vertical 9:16, 5 seconds, single slow lateral tracking shot along a wooden pickup shelf behind a French food shop counter, filled with kraft paper bags, pastry boxes and wrapped parcels, each with a blank kraft tag tied with twine, a small fir garland along the shelf edge, warm morning light. At the end of the move, a hand (navy apron, no face) places one more parcel on the shelf. No readable text, no logos. Photorealistic documentary, fine film grain. Audio: quiet shop, paper, no music, no speech.</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Seedance 2.5 · 9:16 · 5 s · 1080p · audio on</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>60 crédits</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>1, 41, 51</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>V-TEL-NUIT</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Nouveau · Téléphone sur le comptoir la nuit, l'écran s'allume plusieurs fois (commandes qui arrivent)</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>— (texte seul)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Vertical 9:16, 5 seconds, single locked-off close-up. A smartphone lies face up on a wooden shop counter at night in a closed French food shop, blurred Christmas lights glowing in the window behind; the screen lights up softly three times in a row with a plain white glow as notifications arrive, no readable content on the screen. No people, no text, no logos. Photorealistic, fine film grain. Audio: three soft notification chimes, quiet night, no music, no speech.</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Seedance 2.5 · 9:16 · 5 s · 1080p · audio on</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>60 crédits</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>5, 31, 45</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>V-REMISE-NOEL</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Nouveau · Remise d'un paquet de fête par-dessus le comptoir, sourire implicite, rapide</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>— (texte seul)</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Vertical 9:16, 5 seconds, single first-person POV shot at a French food shop counter decorated for Christmas. The shopkeeper's hands (navy apron, chest down, no face) lift a wrapped festive parcel with a blank kraft tag and hand it across the counter toward the camera; the customer's hands take it. Warm morning light, fir garland on the counter edge. No readable text, no logos. Photorealistic documentary. Audio: paper, a short 'merci', shop ambience, no music.</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Seedance 2.5 · 9:16 · 5 s · 1080p · audio on</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>60 crédits</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>27, 43, 55</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>V-QR-SCAN</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Nouveau · Une main scanne le sticker de la vitrine avec son téléphone</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>— (texte seul)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Vertical 9:16, 5 seconds, single close-up shot from the street at dusk. A customer's gloved hand raises a smartphone toward a small blank white square sticker on the glass door of a French food shop decorated for Christmas, holds it still for a second, then lowers the phone; the phone screen shows only a soft plain glow, no readable content. Warm light inside the shop. No faces, no text, no logos. Photorealistic, fine film grain. Audio: street ambience, a soft phone chime, no music, no speech.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Seedance 2.5 · 9:16 · 5 s · 1080p · audio on</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>60 crédits</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>10, 15, 46</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>NW-FRUITSMER</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Mains gantées qui posent la dernière huître, gouttes d'eau</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>c0a50f0f-81f3-4d11-9624-8599eecf3583</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>A fishmonger's hands in blue gloves (no face) place one last oyster on the crushed ice of the platter and add a lemon half, water droplets glisten, very slow top-down drift. Cool bright daylight. No text, no logos. Photorealistic documentary. Audio: ice, quiet shop, no music, no speech.</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Seedance 2.5 · 9:16 · 5 s · 1080p · audio on</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>60 crédits</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>5, 31</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>NW-VOLAILLE</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>La volaille posée sur la balance, l'aiguille se stabilise (vente au poids)</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>aa97dfff-4cef-4441-94db-e3abe8025476</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>A butcher's hands (white coat, no face) lift the trussed poultry on its waxed paper and set it down on a traditional counter scale with a round dial; the needle swings and settles. The dial has no readable numbers. Warm natural light. No text, no logos. Photorealistic documentary. Audio: paper, scale spring, quiet butcher shop, no music, no speech.</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Seedance 2.5 · 9:16 · 5 s · 1080p · audio on</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>60 crédits</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>4, 31</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>NW-COURONNE</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>La fleuriste pose la dernière bougie sur la couronne</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>57b69978-41de-4492-9f2a-e4fe3a966d67</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>A florist's hands (linen apron, no face) press the last white candle into the Advent wreath, adjust a dried orange slice, then step back out of frame. Soft window light, slow top-down drift. No text, no logos. Photorealistic. Audio: greenery rustle, quiet workshop, no music, no speech.</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Seedance 2.5 · 9:16 · 5 s · 1080p · audio on</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>60 crédits</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>9, 49</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>NW-SALLE-6</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>La table de 6 vide : bougies qui vacillent, travelling lent</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>dab06dad-a7b9-45f7-871a-daea60f9c72f</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Slow dolly toward the empty table for six; candle flames flicker, warm pendant lights, other tables softly blurred, nobody sits down. Melancholic stillness. No people, no text, no logos. Photorealistic, fine film grain. Audio: faint restaurant ambience from far away, clock ticking, no music, no speech.</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Seedance 2.5 · 9:16 · 5 s · 1080p · audio on</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>60 crédits</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>29, 47</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>NW-PANIER-FETES</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Mains qui nouent le ruban du panier de fêtes</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>017b0ad6-8ce5-4db2-9af6-ece803391f81</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>A greengrocer's hands (navy apron, no face) tie the red ribbon of the festive fruit basket into a bow and straighten the blank kraft tag, then slide the basket slightly forward on the counter. Warm window light. No text, no logos. Photorealistic documentary. Audio: ribbon, kraft paper, quiet shop, no music, no speech.</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Seedance 2.5 · 9:16 · 5 s · 1080p · audio on</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>60 crédits</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>38, 52</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>V-PIZZA-RUSH</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Nouveau · Boîtes à pizza qui s'empilent au coup de feu de 20 h</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>— (texte seul)</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Vertical 9:16, 5 seconds, single shot at counter height in an Italian pizzeria in the evening rush. A pizzaiolo's hands (white t-shirt, no face) stack plain unprinted kraft pizza boxes one on top of another, quickly, the pile grows to six boxes, the wood-fired oven glowing behind. No readable text, no logos. Photorealistic documentary. Audio: busy kitchen, oven, boxes, no music, no speech.</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Seedance 2.5 · 9:16 · 5 s · 1080p · audio on</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>60 crédits</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>13, 47</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>3 (facultatif)</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>NW-FOODTRUCK</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Food-truck : un sac tendu par la trappe</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>b2cab08c-17be-4588-ab65-f19fcda01bb6</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Slow push-in toward the food truck hatch; a hand inside passes a kraft paper bag through the hatch to a customer seen from behind, the short queue moves forward. Midday light, plane trees. No readable text or logos, no faces. Photorealistic documentary. Audio: market ambience, no music, no speech.</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Seedance 2.5 · 9:16 · 5 s · 1080p · audio on</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>60 crédits</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n"/>
+      <c r="B16" s="2" t="n"/>
+      <c r="C16" s="2" t="n"/>
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n"/>
+      <c r="H16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr"/>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Priorités 1 et 2</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr"/>
+      <c r="G17" s="2">
+        <f>SUMPRODUCT((LEFT(A2:A15,1)&lt;&gt;"3")*60)</f>
+        <v/>
+      </c>
+      <c r="H17" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>